<commit_message>
decompose project voucher to a diffrent files
</commit_message>
<xml_diff>
--- a/yabrov_office_4/storage/exports/Запись_о_документах.xlsx
+++ b/yabrov_office_4/storage/exports/Запись_о_документах.xlsx
@@ -35,9 +35,6 @@
     <t>Пермь</t>
   </si>
   <si>
-    <t>ул. Харченко 16, кв. 376</t>
-  </si>
-  <si>
     <t>ываываыв</t>
   </si>
   <si>
@@ -51,6 +48,9 @@
   </si>
   <si>
     <t>Капернаумова 10, кв. 67</t>
+  </si>
+  <si>
+    <t>пр-т Ленина, д3, кв. 181</t>
   </si>
 </sst>
 </file>
@@ -402,7 +402,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="4.57" bestFit="true" customWidth="true" style="0"/>
@@ -431,10 +431,10 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B2">
-        <v>3915</v>
+        <v>5227</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
@@ -443,109 +443,109 @@
         <v>6</v>
       </c>
       <c r="E2">
-        <v>110.0</v>
+        <v>1870</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B3">
-        <v>2990</v>
+        <v>4726</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E3">
-        <v>1959.99999999999977</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B4">
-        <v>4907</v>
+        <v>4001</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E4">
-        <v>2380.0</v>
+        <v>1925</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B5">
-        <v>1255</v>
+        <v>8615</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E5">
-        <v>2380.0</v>
+        <v>1925</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B6">
-        <v>2456</v>
+        <v>4045</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E6">
-        <v>3075.0</v>
+        <v>1831.50000000000023</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B7">
-        <v>5243</v>
+        <v>6424</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D7" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E7">
-        <v>3075.0</v>
+        <v>2197.80000000000018</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B8">
-        <v>8473</v>
+        <v>2457</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D8" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E8">
-        <v>3075.0</v>
+        <v>2197.80000000000018</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -553,16 +553,16 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>5227</v>
+        <v>9658</v>
       </c>
       <c r="C9" t="s">
         <v>5</v>
       </c>
       <c r="D9" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E9">
-        <v>1870.0</v>
+        <v>1007.60000000000014</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -570,16 +570,16 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>4726</v>
+        <v>3100</v>
       </c>
       <c r="C10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
         <v>8</v>
       </c>
-      <c r="D10" t="s">
-        <v>9</v>
-      </c>
       <c r="E10">
-        <v>1265.0</v>
+        <v>9710.39999999999964</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -587,67 +587,16 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>4001</v>
+        <v>4995</v>
       </c>
       <c r="C11" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E11">
-        <v>1925.0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>8615</v>
-      </c>
-      <c r="C12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12">
-        <v>1925.0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>4045</v>
-      </c>
-      <c r="C13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13">
-        <v>1831.50000000000023</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>6424</v>
-      </c>
-      <c r="C14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14">
-        <v>2197.80000000000018</v>
+        <v>9710.39999999999964</v>
       </c>
     </row>
   </sheetData>

</xml_diff>